<commit_message>
Auto update RUP 24/06/2026  5:00:55,99
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-24).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-24).xlsx
@@ -589,19 +589,19 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1363592000</v>
+        <v>1363719500</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1363592000</v>
+        <v>1363719500</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0</v>
+        <v>127500</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>100</v>
+        <v>100.0093503041966</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Auto update RUP 24/06/2026  8:00:17,40
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-24).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-24).xlsx
@@ -589,19 +589,19 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1363719500</v>
+        <v>1363592000</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1363719500</v>
+        <v>1363592000</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>127500</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>100.0093503041966</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">

</xml_diff>